<commit_message>
Revisi: teks Bahasa Indonesia + update nama tim Duwellduwin, UGM, Victoria/Nayla/Fadhila
</commit_message>
<xml_diff>
--- a/public/excel/MASTER_TOURISM_DATABASE_FINAL.xlsx
+++ b/public/excel/MASTER_TOURISM_DATABASE_FINAL.xlsx
@@ -21,6 +21,8 @@
     <sheet name="11_Accommodation" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="12_Air_Transportation" sheetId="12" state="visible" r:id="rId14"/>
     <sheet name="13_Investment_Potential_Sector" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="14_BCA_Financial_Statements" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="15_Financial_Projection_Model" sheetId="15" state="visible" r:id="rId17"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3250" uniqueCount="941">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3513" uniqueCount="1088">
   <si>
     <t xml:space="preserve">MASTER TOURISM DATABASE — FINAL (V3) — BCA Travel &amp; Tourism Business Case</t>
   </si>
@@ -2521,6 +2523,21 @@
     <t xml:space="preserve">https://ekonomi.bisnis.com/read/20250211/12/1838731/investasi-sektor-hotel-restoran-masih-rendah-bkpm-ungkap-datanya</t>
   </si>
   <si>
+    <t xml:space="preserve">PT Bank Central Asia Tbk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinerja Keuangan BCA dan Entitas Anak Tahun 2024 (Konferensi Pers, 23 Jan 2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.antaranews.com/berita/4604138/bca-dan-entitas-anak-raih-laba-bersih-rp548-triliun-pada-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ketentuan MDR QRIS (Surat Deputi Gubernur BI No. 26/3/KEP.DpG/2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.bi.go.id/id/publikasi/ruang-media/cerita-bi/Pages/mdr-qris.aspx</t>
+  </si>
+  <si>
     <t xml:space="preserve">10 — QA Audit Log</t>
   </si>
   <si>
@@ -2855,6 +2872,432 @@
   </si>
   <si>
     <t xml:space="preserve">Rp15.19 triliun (48.7% of Bali's tourism-sector investment)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 — BCA Official Financial Statements (FY2024, Consolidated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sourced to BCA's own official year-end results press conference (Konferensi Pers Paparan Kinerja BCA, 23 Jan 2025), led by President Director Jahja Setiaatmadja, and cross-verified across multiple independent financial press outlets (Antara, Bisnis.com, Kontan, Bareksa, IPOTNews) that all report identical figures — no discrepancies found. This is a management-disclosed summary, not the full audited financial statements; for line-by-line audited figures see BCA's Annual Report 2024 (IDX filing) linked in the last row below. Figures are for BCA and consolidated subsidiaries.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Income Statement — FY2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YoY Growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net Interest Income (NII)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp82.3 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+9.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT Bank Central Asia Tbk (BCA) — Konferensi Pers Paparan Kinerja BCA, 23 Januari 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinerja Keuangan BCA dan Entitas Anak Tahun 2024 (Audited, Consolidated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-Interest Income (fee-based)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp25.2 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+10.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Operating Income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp107.4 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+9.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provision Expense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp2 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net Profit (BCA + Subsidiaries)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp54.8 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp48.6 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+12.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credit Portfolio / Balance Sheet — as of December 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of Total Credit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Credit Disbursed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp922 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+13.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— Corporate Credit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp426.8 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+15.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— Commercial Credit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp137.9 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+8.9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— SME (UKM) Credit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp123.8 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+14.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— Consumer Credit (total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp223.7 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+12.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    — Vehicle Loans (KKB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp65.3 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    — Mortgage (KPR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp135.5 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+11.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    — Other Consumer (incl. credit card)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp22.9 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+12.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sustainable-Sector Lending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp229 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+12.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASA (Current Account + Savings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp924 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+4.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82% of total DPK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total DPK (Third-Party Funds)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp1,134 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+2.9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Assets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp1,449.3 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vs Rp1,408.1T (2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-Performing Loan (NPL) ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan at Risk (LAR) ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">improved from 6.9% (2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total customer accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41+ juta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total transaction frequency (all channels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36 miliar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+21%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile + internet banking transaction frequency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.6 miliar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+24%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full audited financial statements (line-by-line)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Available as official filing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT Bank Central Asia Tbk / Indonesia Stock Exchange (IDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laporan Tahunan 2024 (Annual Report, IDX filing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 — Financial Projection Model (QRIS Tourism-Corridor Opportunity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMPORTANT — read before using this sheet. This is a MODEL, not official data. Every row is tagged either OFFICIAL INPUT (a real, sourced, regulated or published figure) or TEAM ASSUMPTION (a judgment call this team is making, clearly separated so it can be challenged or changed). No official publication states what share of QRIS fee revenue BCA specifically captures per province — that split across acquirers/issuers is not publicly disclosed by BI or BCA, so this model does NOT invent one number. Instead it computes the TOTAL addressable QRIS fee pool from official inputs, then shows BCA's revenue under three explicit market-share scenarios (Low/Base/High) so the reader judges the assumption, not us.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 1 — Official Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRIS MDR — Usaha Mikro (UMI), transactions &gt; Rp500,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFFICIAL INPUT (regulated rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Deputi Gubernur BI No. 26/3/KEP.DpG/2024; RDG Februari 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRIS MDR — Usaha Kecil/Menengah/Besar (UKE/UME/UBE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National QRIS transaction value, Semester I 2025 (cumulative)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rp579 triliun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFFICIAL INPUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siaran Pers QRIS Jelajah Indonesia 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National domestic trip growth, Jan-Jun 2025 vs 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+17.70%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kementerian Pariwisata RI (diolah dari BPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perjalanan Wisnus Menurut Provinsi Asal 2024-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-growth province trip growth (avg. of provinces &gt;30% growth, this workbook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See 04_Province_Domestic_Trips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFFICIAL INPUT (derived from BPS data already in this workbook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BPS / Kementerian Pariwisata RI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 2 — Team Assumptions (explicitly NOT official data)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low Case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base Case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High Case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale (team judgment, not sourced)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BCA's share of QRIS merchant acquiring in target tourism provinces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BCA is a top-3 acquirer nationally by transaction value (per public commentary) but does not disclose a province-level or category-level QRIS acquiring market share; this range reflects a conservative-to-optimistic spread a team would need to validate with BCA directly before using in a real business case.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incremental tourism-driven QRIS volume growth, target provinces (annualized)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchored to this workbook's real high-growth-province trip data (many provinces already show +40-120% Jan-Jun trip growth), discounted down because trip growth != QRIS volume growth 1:1 — assumption, not measured.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 3 — Resulting Addressable Revenue Range (calculated, not official)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed BCA Acquiring Share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed Incremental QRIS Growth (Tourism Corridor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illustrative Annual Revenue Range for BCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tens of billions of Rupiah (low single-digit % of BCA's Rp25.2T non-interest income)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conservative: small share of a modest incremental slice of the national Rp579T semester QRIS pool, blended MDR ~0.3-0.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low hundreds of billions of Rupiah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mid-range assumption; still under 1% of BCA's total FY2024 non-interest income (Rp25.2T) — directionally material but not transformative on its own</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Several hundred billion Rupiah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimistic case assuming aggressive, successful merchant-acquisition execution in tourism corridors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read this table as an ORDER-OF-MAGNITUDE framework for discussion, not a forecast to quote as fact. The precise Rupiah figures are intentionally left as ranges/descriptions rather than single numbers, because presenting false precision from an admittedly assumption-driven model would misrepresent it as official data. If BCA's actual QRIS acquiring economics become available, replace Step 2's assumptions and this table recalculates automatically in spirit (manually update the range descriptions).</t>
   </si>
 </sst>
 </file>
@@ -2866,7 +3309,7 @@
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.00\%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2938,6 +3381,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF1F6B3A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -3030,7 +3481,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3131,6 +3582,14 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3151,7 +3610,7 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF1F6B3A"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF9C6500"/>
       <rgbColor rgb="FF800080"/>
@@ -3581,97 +4040,97 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
     </row>
   </sheetData>
@@ -3706,7 +4165,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3717,7 +4176,7 @@
     </row>
     <row r="2" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -3728,7 +4187,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3754,10 +4213,10 @@
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>470</v>
@@ -3775,10 +4234,10 @@
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>470</v>
@@ -3796,10 +4255,10 @@
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>470</v>
@@ -3817,10 +4276,10 @@
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>470</v>
@@ -3838,10 +4297,10 @@
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>470</v>
@@ -3859,10 +4318,10 @@
     </row>
     <row r="11" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>470</v>
@@ -3880,10 +4339,10 @@
     </row>
     <row r="12" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>470</v>
@@ -3901,10 +4360,10 @@
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>470</v>
@@ -3922,10 +4381,10 @@
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>470</v>
@@ -3943,10 +4402,10 @@
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>470</v>
@@ -3964,10 +4423,10 @@
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>470</v>
@@ -3985,10 +4444,10 @@
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>470</v>
@@ -4006,10 +4465,10 @@
     </row>
     <row r="18" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>470</v>
@@ -4027,7 +4486,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4035,10 +4494,10 @@
         <v>188</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>19</v>
@@ -4062,7 +4521,7 @@
         <v>3125</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>816</v>
@@ -4083,7 +4542,7 @@
         <v>4154</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>816</v>
@@ -4102,7 +4561,7 @@
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="8" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>816</v>
@@ -4123,7 +4582,7 @@
         <v>2279</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>816</v>
@@ -4144,7 +4603,7 @@
         <v>4055</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>816</v>
@@ -4165,7 +4624,7 @@
         <v>2000</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>816</v>
@@ -4184,7 +4643,7 @@
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="8" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>816</v>
@@ -4203,7 +4662,7 @@
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="6" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>816</v>
@@ -4222,7 +4681,7 @@
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="8" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>816</v>
@@ -4241,7 +4700,7 @@
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="6" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>816</v>
@@ -4252,9 +4711,9 @@
       <c r="G31" s="7"/>
     </row>
     <row r="32" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4262,10 +4721,10 @@
         <v>188</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>19</v>
@@ -4286,7 +4745,7 @@
         <v>2.74</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>818</v>
@@ -4307,7 +4766,7 @@
         <v>2.44</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>818</v>
@@ -4328,7 +4787,7 @@
         <v>2.3</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>818</v>
@@ -4349,7 +4808,7 @@
         <v>2.24</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>818</v>
@@ -4370,7 +4829,7 @@
         <v>1.97</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>818</v>
@@ -4479,9 +4938,9 @@
       <c r="G44" s="7"/>
     </row>
     <row r="45" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="22" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4495,7 +4954,7 @@
         <v>456</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>457</v>
@@ -4507,25 +4966,25 @@
     </row>
     <row r="48" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="23" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="C48" s="24" t="s">
         <v>470</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="F48" s="23" t="s">
         <v>823</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4562,7 +5021,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4572,7 +5031,7 @@
     </row>
     <row r="2" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -4602,50 +5061,50 @@
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>794</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>794</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>762</v>
@@ -4654,18 +5113,18 @@
         <v>794</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>762</v>
@@ -4674,58 +5133,58 @@
         <v>794</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>794</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>794</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>470</v>
@@ -4773,7 +5232,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4783,7 +5242,7 @@
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -4813,19 +5272,19 @@
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>826</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>828</v>
@@ -4833,19 +5292,19 @@
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>826</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>828</v>
@@ -4853,19 +5312,19 @@
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>826</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>828</v>
@@ -4873,19 +5332,19 @@
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>826</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>828</v>
@@ -4893,19 +5352,19 @@
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>826</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>828</v>
@@ -4913,19 +5372,19 @@
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>826</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>828</v>
@@ -4933,19 +5392,19 @@
     </row>
     <row r="11" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>826</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>828</v>
@@ -4955,6 +5414,955 @@
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>946</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>947</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>949</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>767</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>950</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>951</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>952</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>953</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>954</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>957</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>958</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>959</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>960</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>961</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>962</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>963</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>964</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>965</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>966</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>967</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>968</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>949</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>951</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>970</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>971</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>972</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>973</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>974</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>975</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>977</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>978</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>979</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>980</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>981</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>982</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>983</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>984</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>985</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>986</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>987</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>988</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>989</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>990</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>991</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>992</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>985</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>993</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>994</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>995</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>996</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>997</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>998</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>999</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>1008</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>1015</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>956</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>1031</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>1032</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>782</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>1041</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>1041</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>1047</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>1050</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>1051</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>1055</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>1051</v>
+      </c>
+      <c r="F10" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="22" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>1058</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>1060</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>1061</v>
+      </c>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>1064</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>1065</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>1070</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>1073</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>1075</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>1076</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>1079</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>1070</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A23:F23"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16025,7 +17433,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -16295,7 +17703,7 @@
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="n">
         <v>15</v>
       </c>
@@ -16312,7 +17720,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="n">
         <v>16</v>
       </c>
@@ -16329,7 +17737,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="n">
         <v>17</v>
       </c>
@@ -16346,7 +17754,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="n">
         <v>18</v>
       </c>
@@ -16363,7 +17771,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="n">
         <v>19</v>
       </c>
@@ -16378,6 +17786,40 @@
       </c>
       <c r="E21" s="6" t="s">
         <v>828</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>829</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>830</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>509</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>832</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>